<commit_message>
COMPLETED: Homepage and How it Works Page; TODO: Complete Try It Page
</commit_message>
<xml_diff>
--- a/Data IBIS/11111CA Soybean Farming in Canada Industry Report (1).xlsx
+++ b/Data IBIS/11111CA Soybean Farming in Canada Industry Report (1).xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\awe50\Desktop\Projects Deployment\Western AI\WAI\Data IBIS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E6B79B-92B8-45C1-9E61-BDDC67CF8A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Annual Change" sheetId="1" r:id="rId1"/>
@@ -52,15 +58,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -86,16 +92,20 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -397,15 +407,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" customWidth="1" style="1"/>
+    <col min="1" max="1" width="9.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="12.77734375" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -440,12 +459,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>2006</v>
       </c>
       <c r="B2" s="2">
-        <v>-20.33</v>
+        <v>-20.329999999999998</v>
       </c>
       <c r="C2" s="2">
         <v>-15.76</v>
@@ -469,13 +488,13 @@
         <v>-25.97</v>
       </c>
       <c r="J2" s="2">
-        <v>-31.859000</v>
+        <v>-31.859000000000002</v>
       </c>
       <c r="K2" s="2">
         <v>-2.56</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2007</v>
       </c>
@@ -483,10 +502,10 @@
         <v>27.82</v>
       </c>
       <c r="C3" s="2">
-        <v>4.60</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="D3" s="2">
-        <v>6.90</v>
+        <v>6.9</v>
       </c>
       <c r="E3" s="2">
         <v>6.87</v>
@@ -495,22 +514,22 @@
         <v>14.13</v>
       </c>
       <c r="G3" s="2">
-        <v>39.62</v>
+        <v>39.619999999999997</v>
       </c>
       <c r="H3" s="2">
-        <v>-19.06</v>
+        <v>-19.059999999999999</v>
       </c>
       <c r="I3" s="2">
         <v>16.63</v>
       </c>
       <c r="J3" s="2">
-        <v>16.470800</v>
+        <v>16.470800000000001</v>
       </c>
       <c r="K3" s="2">
         <v>45.92</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2008</v>
       </c>
@@ -533,19 +552,19 @@
         <v>25.55</v>
       </c>
       <c r="H4" s="2">
-        <v>150.89</v>
+        <v>150.88999999999999</v>
       </c>
       <c r="I4" s="2">
         <v>-13.01</v>
       </c>
       <c r="J4" s="2">
-        <v>-14.750200</v>
+        <v>-14.7502</v>
       </c>
       <c r="K4" s="2">
         <v>42.74</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2009</v>
       </c>
@@ -553,16 +572,16 @@
         <v>28.19</v>
       </c>
       <c r="C5" s="2">
-        <v>17.19</v>
+        <v>17.190000000000001</v>
       </c>
       <c r="D5" s="2">
         <v>3.06</v>
       </c>
       <c r="E5" s="2">
-        <v>3.10</v>
+        <v>3.1</v>
       </c>
       <c r="F5" s="2">
-        <v>26.40</v>
+        <v>26.4</v>
       </c>
       <c r="G5" s="2">
         <v>13.55</v>
@@ -574,13 +593,13 @@
         <v>32.79</v>
       </c>
       <c r="J5" s="2">
-        <v>38.812600</v>
+        <v>38.812600000000003</v>
       </c>
       <c r="K5" s="2">
         <v>-16.43</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>2010</v>
       </c>
@@ -597,30 +616,30 @@
         <v>5.27</v>
       </c>
       <c r="F6" s="2">
-        <v>11.90</v>
+        <v>11.9</v>
       </c>
       <c r="G6" s="2">
-        <v>30.30</v>
+        <v>30.3</v>
       </c>
       <c r="H6" s="2">
-        <v>-43.00</v>
+        <v>-43</v>
       </c>
       <c r="I6" s="2">
         <v>22.51</v>
       </c>
       <c r="J6" s="2">
-        <v>-8.445000</v>
+        <v>-8.4450000000000003</v>
       </c>
       <c r="K6" s="2">
         <v>1.69</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>2011</v>
       </c>
       <c r="B7" s="2">
-        <v>-8.54</v>
+        <v>-8.5399999999999991</v>
       </c>
       <c r="C7" s="2">
         <v>-11.55</v>
@@ -641,16 +660,16 @@
         <v>32.24</v>
       </c>
       <c r="I7" s="2">
-        <v>-17.40</v>
+        <v>-17.399999999999999</v>
       </c>
       <c r="J7" s="2">
-        <v>-15.595000</v>
+        <v>-15.595000000000001</v>
       </c>
       <c r="K7" s="2">
         <v>25.79</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>2012</v>
       </c>
@@ -658,7 +677,7 @@
         <v>51.65</v>
       </c>
       <c r="C8" s="2">
-        <v>56.10</v>
+        <v>56.1</v>
       </c>
       <c r="D8" s="2">
         <v>24.37</v>
@@ -679,13 +698,13 @@
         <v>52.51</v>
       </c>
       <c r="J8" s="2">
-        <v>53.423800</v>
+        <v>53.4238</v>
       </c>
       <c r="K8" s="2">
         <v>11.05</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>2013</v>
       </c>
@@ -699,7 +718,7 @@
         <v>2.72</v>
       </c>
       <c r="E9" s="2">
-        <v>2.70</v>
+        <v>2.7</v>
       </c>
       <c r="F9" s="2">
         <v>8.01</v>
@@ -714,13 +733,13 @@
         <v>6.98</v>
       </c>
       <c r="J9" s="2">
-        <v>12.527800</v>
+        <v>12.527799999999999</v>
       </c>
       <c r="K9" s="2">
         <v>-3.83</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>2014</v>
       </c>
@@ -728,16 +747,16 @@
         <v>-9.64</v>
       </c>
       <c r="C10" s="2">
-        <v>-15.50</v>
+        <v>-15.5</v>
       </c>
       <c r="D10" s="2">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="E10" s="2">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="F10" s="2">
-        <v>-9.13</v>
+        <v>-9.1300000000000008</v>
       </c>
       <c r="G10" s="2">
         <v>-7.53</v>
@@ -749,13 +768,13 @@
         <v>-6.53</v>
       </c>
       <c r="J10" s="2">
-        <v>-7.978300</v>
+        <v>-7.9782999999999999</v>
       </c>
       <c r="K10" s="2">
         <v>-11.49</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>2015</v>
       </c>
@@ -781,16 +800,16 @@
         <v>-5.21</v>
       </c>
       <c r="I11" s="2">
-        <v>-2.20</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="J11" s="2">
-        <v>-36.631300</v>
+        <v>-36.631300000000003</v>
       </c>
       <c r="K11" s="2">
         <v>-24.13</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>2016</v>
       </c>
@@ -801,7 +820,7 @@
         <v>21.32</v>
       </c>
       <c r="D12" s="2">
-        <v>-6.30</v>
+        <v>-6.3</v>
       </c>
       <c r="E12" s="2">
         <v>-6.28</v>
@@ -819,13 +838,13 @@
         <v>19.48</v>
       </c>
       <c r="J12" s="2">
-        <v>31.190700</v>
+        <v>31.1907</v>
       </c>
       <c r="K12" s="2">
         <v>4.41</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>2017</v>
       </c>
@@ -836,7 +855,7 @@
         <v>-11.01</v>
       </c>
       <c r="D13" s="2">
-        <v>39.63</v>
+        <v>39.630000000000003</v>
       </c>
       <c r="E13" s="2">
         <v>39.61</v>
@@ -854,21 +873,21 @@
         <v>1.67</v>
       </c>
       <c r="J13" s="2">
-        <v>13.319600</v>
+        <v>13.319599999999999</v>
       </c>
       <c r="K13" s="2">
         <v>-1.08</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>2018</v>
       </c>
       <c r="B14" s="2">
-        <v>0.20</v>
+        <v>0.2</v>
       </c>
       <c r="C14" s="2">
-        <v>9.90</v>
+        <v>9.9</v>
       </c>
       <c r="D14" s="2">
         <v>-1.34</v>
@@ -889,13 +908,13 @@
         <v>3.63</v>
       </c>
       <c r="J14" s="2">
-        <v>-9.513300</v>
+        <v>-9.5132999999999992</v>
       </c>
       <c r="K14" s="2">
         <v>-4.55</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>2019</v>
       </c>
@@ -909,7 +928,7 @@
         <v>-6.31</v>
       </c>
       <c r="E15" s="2">
-        <v>-6.30</v>
+        <v>-6.3</v>
       </c>
       <c r="F15" s="2">
         <v>-17.14</v>
@@ -924,13 +943,13 @@
         <v>-14.34</v>
       </c>
       <c r="J15" s="2">
-        <v>-0.148800</v>
+        <v>-0.14879999999999999</v>
       </c>
       <c r="K15" s="2">
         <v>-4.54</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>2020</v>
       </c>
@@ -947,7 +966,7 @@
         <v>-2.63</v>
       </c>
       <c r="F16" s="2">
-        <v>2.60</v>
+        <v>2.6</v>
       </c>
       <c r="G16" s="2">
         <v>23.63</v>
@@ -959,13 +978,13 @@
         <v>3.27</v>
       </c>
       <c r="J16" s="2">
-        <v>-27.896200</v>
+        <v>-27.8962</v>
       </c>
       <c r="K16" s="2">
         <v>6.99</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>2021</v>
       </c>
@@ -979,28 +998,28 @@
         <v>6.48</v>
       </c>
       <c r="E17" s="2">
-        <v>6.20</v>
+        <v>6.2</v>
       </c>
       <c r="F17" s="2">
         <v>7.23</v>
       </c>
       <c r="G17" s="2">
-        <v>8.45</v>
+        <v>8.4499999999999993</v>
       </c>
       <c r="H17" s="2">
-        <v>20.17</v>
+        <v>20.170000000000002</v>
       </c>
       <c r="I17" s="2">
         <v>7.91</v>
       </c>
       <c r="J17" s="2">
-        <v>17.781700</v>
+        <v>17.781700000000001</v>
       </c>
       <c r="K17" s="2">
         <v>13.53</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>2022</v>
       </c>
@@ -1014,28 +1033,28 @@
         <v>4.12</v>
       </c>
       <c r="E18" s="2">
-        <v>4.15</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="F18" s="2">
         <v>3.03</v>
       </c>
       <c r="G18" s="2">
-        <v>4.11</v>
+        <v>4.1100000000000003</v>
       </c>
       <c r="H18" s="2">
-        <v>2.22</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="I18" s="2">
         <v>3.13</v>
       </c>
       <c r="J18" s="2">
-        <v>2.584800</v>
+        <v>2.5848</v>
       </c>
       <c r="K18" s="2">
         <v>-0.64</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>2023</v>
       </c>
@@ -1055,22 +1074,22 @@
         <v>2.09</v>
       </c>
       <c r="G19" s="2">
-        <v>2.03</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="H19" s="2">
-        <v>1.12</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="I19" s="2">
         <v>2.06</v>
       </c>
       <c r="J19" s="2">
-        <v>1.308100</v>
+        <v>1.3081</v>
       </c>
       <c r="K19" s="2">
         <v>0.02</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>2024</v>
       </c>
@@ -1084,10 +1103,10 @@
         <v>3.91</v>
       </c>
       <c r="E20" s="2">
-        <v>4.14</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="F20" s="2">
-        <v>1.10</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G20" s="2">
         <v>0.78</v>
@@ -1099,13 +1118,13 @@
         <v>1.01</v>
       </c>
       <c r="J20" s="2">
-        <v>0.234700</v>
+        <v>0.23469999999999999</v>
       </c>
       <c r="K20" s="2">
         <v>-0.22</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>2025</v>
       </c>
@@ -1116,10 +1135,10 @@
         <v>1.64</v>
       </c>
       <c r="D21" s="2">
-        <v>1.10</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E21" s="2">
-        <v>1.10</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F21" s="2">
         <v>0.94</v>
@@ -1131,16 +1150,16 @@
         <v>0.72</v>
       </c>
       <c r="I21" s="2">
-        <v>1.00</v>
+        <v>1</v>
       </c>
       <c r="J21" s="2">
-        <v>0.849000</v>
+        <v>0.84899999999999998</v>
       </c>
       <c r="K21" s="2">
         <v>0.35</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>2026</v>
       </c>
@@ -1160,7 +1179,7 @@
         <v>0.86</v>
       </c>
       <c r="G22" s="2">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="H22" s="2">
         <v>0.42</v>
@@ -1169,13 +1188,13 @@
         <v>0.86</v>
       </c>
       <c r="J22" s="2">
-        <v>0.602400</v>
+        <v>0.60240000000000005</v>
       </c>
       <c r="K22" s="2">
         <v>2.61</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>2027</v>
       </c>
@@ -1204,14 +1223,14 @@
         <v>1.23</v>
       </c>
       <c r="J23" s="2">
-        <v>0.382300</v>
+        <v>0.38229999999999997</v>
       </c>
       <c r="K23" s="2">
         <v>0.42</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup orientation="portrait" scale="100" paperSize="9" fitToWidth="0" fitToHeight="0" horizontalDpi="0" verticalDpi="0" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>